<commit_message>
extracted new pf results; changed ppc branch type to float; changed values for zero sequence parameters of wp2.3
</commit_message>
<xml_diff>
--- a/pandapower/test/shortcircuit/sce_tests/sc_result_comparison/wp_2.3/10_eight_bus_radial_grid_2ph_dd_MP_pf_sc_results_0_bus.xlsx
+++ b/pandapower/test/shortcircuit/sce_tests/sc_result_comparison/wp_2.3/10_eight_bus_radial_grid_2ph_dd_MP_pf_sc_results_0_bus.xlsx
@@ -68,10 +68,13 @@
     <t>pf_va_degree</t>
   </si>
   <si>
-    <t>Bus_0</t>
+    <t>Bus_1</t>
   </si>
   <si>
-    <t>Bus_1</t>
+    <t>Bus_5_3-1ph</t>
+  </si>
+  <si>
+    <t>Bus_6_3-1ph</t>
   </si>
   <si>
     <t>Bus_2_3-2ph</t>
@@ -83,10 +86,7 @@
     <t>Bus_4_3-2ph</t>
   </si>
   <si>
-    <t>Bus_5_3-1ph</t>
-  </si>
-  <si>
-    <t>Bus_6_3-1ph</t>
+    <t>Bus_0</t>
   </si>
   <si>
     <t>Bus_7_3-1ph</t>
@@ -535,22 +535,22 @@
         <v>7</v>
       </c>
       <c r="B2">
-        <v>2.886751509919007</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>100.0000056801178</v>
+        <v>0</v>
       </c>
       <c r="D2">
-        <v>0.4378163589895365</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>4.378163482065627</v>
+        <v>0</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2">
-        <v>84.2894067227804</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -673,22 +673,22 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>2.886751509919007</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>100.0000056801178</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>0.4378163589895365</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>4.378163482065627</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>84.2894067227804</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -785,7 +785,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -844,7 +844,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -903,7 +903,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -962,7 +962,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1080,7 +1080,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1139,7 +1139,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1326,7 +1326,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1385,7 +1385,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1444,7 +1444,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -1503,7 +1503,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1562,7 +1562,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1621,7 +1621,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -1680,7 +1680,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1867,7 +1867,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -1926,7 +1926,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -1985,7 +1985,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2044,7 +2044,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2103,7 +2103,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2162,7 +2162,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2221,7 +2221,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2408,7 +2408,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2467,7 +2467,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2526,7 +2526,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2585,7 +2585,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -2644,7 +2644,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -2703,7 +2703,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2762,7 +2762,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2949,7 +2949,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -3008,7 +3008,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -3067,7 +3067,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3126,7 +3126,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3185,7 +3185,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -3244,7 +3244,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -3490,7 +3490,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -3549,7 +3549,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -3608,7 +3608,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -3667,7 +3667,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -3726,7 +3726,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -3785,7 +3785,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3844,7 +3844,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -4031,7 +4031,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -4149,7 +4149,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -4208,7 +4208,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -4267,7 +4267,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -4326,7 +4326,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -4385,7 +4385,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -4575,7 +4575,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.881446570267198</v>
@@ -4637,7 +4637,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -4699,7 +4699,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -4761,7 +4761,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -4823,7 +4823,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -4885,7 +4885,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -4947,7 +4947,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -5143,7 +5143,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.881446570267198</v>
@@ -5205,7 +5205,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -5267,7 +5267,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -5329,7 +5329,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -5391,7 +5391,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -5453,7 +5453,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -5515,7 +5515,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -5711,7 +5711,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.170838853958249</v>
@@ -5773,7 +5773,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -5835,7 +5835,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -5897,7 +5897,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -5959,7 +5959,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -6021,7 +6021,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -6083,7 +6083,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -6240,7 +6240,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.886751509919005</v>
@@ -6263,7 +6263,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -6286,7 +6286,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -6309,7 +6309,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -6332,7 +6332,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -6355,7 +6355,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -6378,7 +6378,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -6496,7 +6496,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.170838853958249</v>
@@ -6558,7 +6558,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -6620,7 +6620,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -6682,7 +6682,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -6744,7 +6744,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -6806,7 +6806,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -6868,7 +6868,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -7064,7 +7064,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.304577936611224</v>
@@ -7126,7 +7126,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -7188,7 +7188,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -7250,7 +7250,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -7312,7 +7312,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -7374,7 +7374,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -7436,7 +7436,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -7632,7 +7632,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.304577936611224</v>
@@ -7694,7 +7694,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -7756,7 +7756,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -7818,7 +7818,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -7880,7 +7880,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -7942,7 +7942,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -8004,7 +8004,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -8200,7 +8200,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.012909147793288</v>
@@ -8262,7 +8262,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -8324,7 +8324,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -8386,7 +8386,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -8448,7 +8448,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -8510,7 +8510,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -8572,7 +8572,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -8768,7 +8768,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.012909147793288</v>
@@ -8830,7 +8830,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -8892,7 +8892,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -8954,7 +8954,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -9016,7 +9016,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -9078,7 +9078,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -9140,7 +9140,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -9336,7 +9336,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -9398,7 +9398,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -9460,7 +9460,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -9522,7 +9522,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -9584,7 +9584,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -9646,7 +9646,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -9708,7 +9708,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -9904,7 +9904,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -9966,7 +9966,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -10028,7 +10028,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -10090,7 +10090,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -10152,7 +10152,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -10214,7 +10214,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -10276,7 +10276,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -10472,7 +10472,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -10534,7 +10534,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -10596,7 +10596,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -10658,7 +10658,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -10720,7 +10720,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -10782,7 +10782,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -10844,7 +10844,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -11040,7 +11040,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -11102,7 +11102,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -11164,7 +11164,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -11226,7 +11226,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -11288,7 +11288,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -11350,7 +11350,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -11412,7 +11412,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -11608,7 +11608,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -11670,7 +11670,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -11732,7 +11732,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -11794,7 +11794,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -11856,7 +11856,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -11918,7 +11918,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -11980,7 +11980,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -12137,7 +12137,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.171673335390809</v>
@@ -12160,7 +12160,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -12183,7 +12183,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -12206,7 +12206,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -12229,7 +12229,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -12252,7 +12252,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -12275,7 +12275,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -12393,7 +12393,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -12455,7 +12455,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -12517,7 +12517,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -12579,7 +12579,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -12641,7 +12641,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -12703,7 +12703,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -12765,7 +12765,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -12961,7 +12961,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -13023,7 +13023,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -13085,7 +13085,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -13147,7 +13147,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -13209,7 +13209,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -13271,7 +13271,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -13333,7 +13333,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -13529,7 +13529,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -13591,7 +13591,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -13653,7 +13653,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -13715,7 +13715,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -13777,7 +13777,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -13839,7 +13839,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -13901,7 +13901,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -14058,7 +14058,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.171673335390809</v>
@@ -14081,7 +14081,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -14104,7 +14104,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -14127,7 +14127,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -14150,7 +14150,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -14173,7 +14173,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -14196,7 +14196,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -14275,7 +14275,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.309401157911545</v>
@@ -14298,7 +14298,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -14321,7 +14321,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -14344,7 +14344,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -14367,7 +14367,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -14390,7 +14390,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -14413,7 +14413,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -14492,7 +14492,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>2.309401157911545</v>
@@ -14515,7 +14515,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -14538,7 +14538,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -14561,7 +14561,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -14584,7 +14584,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -14607,7 +14607,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -14630,7 +14630,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -14709,7 +14709,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.013804257465359</v>
@@ -14732,7 +14732,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -14755,7 +14755,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -14778,7 +14778,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -14801,7 +14801,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -14824,7 +14824,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -14847,7 +14847,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -14926,7 +14926,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1.013804257465359</v>
@@ -14949,7 +14949,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -14972,7 +14972,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -14995,7 +14995,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -15018,7 +15018,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -15041,7 +15041,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -15064,7 +15064,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -15179,7 +15179,7 @@
     </row>
     <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -15238,7 +15238,7 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -15297,7 +15297,7 @@
     </row>
     <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -15356,7 +15356,7 @@
     </row>
     <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -15415,7 +15415,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -15474,7 +15474,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -15533,7 +15533,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>0</v>

</xml_diff>